<commit_message>
Agregando Logica de Movimientos De Inventario
</commit_message>
<xml_diff>
--- a/Planificacion/Base De Datos.xlsx
+++ b/Planificacion/Base De Datos.xlsx
@@ -8,24 +8,35 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rayke\Documents\Programacion Web\Programacion 3\Proyecto Final\Reto-3-Grupo-J\Planificacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B40294D-C262-4201-8894-A7443C4D2EFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EC88281-F348-415D-BE5A-62A860755B20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="80">
   <si>
     <t>role_id</t>
   </si>
@@ -262,6 +273,9 @@
   </si>
   <si>
     <t>password_hash</t>
+  </si>
+  <si>
+    <t>int8</t>
   </si>
 </sst>
 </file>
@@ -444,6 +458,15 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -457,15 +480,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -761,15 +775,15 @@
   </cols>
   <sheetData>
     <row r="2" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D2" s="16" t="s">
+      <c r="D2" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
-      <c r="H2" s="16"/>
-      <c r="I2" s="16"/>
-      <c r="J2" s="16"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="11"/>
+      <c r="J2" s="11"/>
     </row>
     <row r="3" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D3" s="2" t="s">
@@ -857,15 +871,15 @@
       </c>
     </row>
     <row r="9" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D9" s="17" t="s">
+      <c r="D9" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17"/>
-      <c r="H9" s="17"/>
-      <c r="I9" s="17"/>
-      <c r="J9" s="17"/>
+      <c r="E9" s="12"/>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="12"/>
+      <c r="I9" s="12"/>
+      <c r="J9" s="12"/>
     </row>
     <row r="10" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D10" s="2" t="s">
@@ -1017,15 +1031,15 @@
       </c>
     </row>
     <row r="20" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D20" s="10" t="s">
+      <c r="D20" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="E20" s="10"/>
-      <c r="F20" s="10"/>
-      <c r="G20" s="10"/>
-      <c r="H20" s="10"/>
-      <c r="I20" s="10"/>
-      <c r="J20" s="10"/>
+      <c r="E20" s="13"/>
+      <c r="F20" s="13"/>
+      <c r="G20" s="13"/>
+      <c r="H20" s="13"/>
+      <c r="I20" s="13"/>
+      <c r="J20" s="13"/>
     </row>
     <row r="21" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D21" s="2" t="s">
@@ -1171,15 +1185,15 @@
       </c>
     </row>
     <row r="31" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D31" s="11" t="s">
+      <c r="D31" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="E31" s="11"/>
-      <c r="F31" s="11"/>
-      <c r="G31" s="11"/>
-      <c r="H31" s="11"/>
-      <c r="I31" s="11"/>
-      <c r="J31" s="11"/>
+      <c r="E31" s="14"/>
+      <c r="F31" s="14"/>
+      <c r="G31" s="14"/>
+      <c r="H31" s="14"/>
+      <c r="I31" s="14"/>
+      <c r="J31" s="14"/>
     </row>
     <row r="32" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D32" s="2" t="s">
@@ -1391,15 +1405,15 @@
       </c>
     </row>
     <row r="46" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D46" s="12" t="s">
+      <c r="D46" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="E46" s="12"/>
-      <c r="F46" s="12"/>
-      <c r="G46" s="12"/>
-      <c r="H46" s="12"/>
-      <c r="I46" s="12"/>
-      <c r="J46" s="12"/>
+      <c r="E46" s="15"/>
+      <c r="F46" s="15"/>
+      <c r="G46" s="15"/>
+      <c r="H46" s="15"/>
+      <c r="I46" s="15"/>
+      <c r="J46" s="15"/>
     </row>
     <row r="47" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D47" s="2" t="s">
@@ -1429,7 +1443,7 @@
         <v>46</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>7</v>
+        <v>79</v>
       </c>
       <c r="F48" s="1" t="s">
         <v>36</v>
@@ -1579,15 +1593,15 @@
       </c>
     </row>
     <row r="59" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D59" s="13" t="s">
+      <c r="D59" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="E59" s="13"/>
-      <c r="F59" s="13"/>
-      <c r="G59" s="13"/>
-      <c r="H59" s="13"/>
-      <c r="I59" s="13"/>
-      <c r="J59" s="13"/>
+      <c r="E59" s="16"/>
+      <c r="F59" s="16"/>
+      <c r="G59" s="16"/>
+      <c r="H59" s="16"/>
+      <c r="I59" s="16"/>
+      <c r="J59" s="16"/>
     </row>
     <row r="60" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D60" s="2" t="s">
@@ -1752,15 +1766,15 @@
       </c>
     </row>
     <row r="71" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D71" s="14" t="s">
+      <c r="D71" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="E71" s="14"/>
-      <c r="F71" s="14"/>
-      <c r="G71" s="14"/>
-      <c r="H71" s="14"/>
-      <c r="I71" s="14"/>
-      <c r="J71" s="14"/>
+      <c r="E71" s="17"/>
+      <c r="F71" s="17"/>
+      <c r="G71" s="17"/>
+      <c r="H71" s="17"/>
+      <c r="I71" s="17"/>
+      <c r="J71" s="17"/>
     </row>
     <row r="72" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D72" s="2" t="s">
@@ -1790,7 +1804,7 @@
         <v>59</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>7</v>
+        <v>79</v>
       </c>
       <c r="F73" s="1" t="s">
         <v>36</v>
@@ -1975,15 +1989,15 @@
       </c>
     </row>
     <row r="87" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D87" s="15" t="s">
+      <c r="D87" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="E87" s="15"/>
-      <c r="F87" s="15"/>
-      <c r="G87" s="15"/>
-      <c r="H87" s="15"/>
-      <c r="I87" s="15"/>
-      <c r="J87" s="15"/>
+      <c r="E87" s="10"/>
+      <c r="F87" s="10"/>
+      <c r="G87" s="10"/>
+      <c r="H87" s="10"/>
+      <c r="I87" s="10"/>
+      <c r="J87" s="10"/>
     </row>
     <row r="88" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D88" s="2" t="s">
@@ -2013,7 +2027,7 @@
         <v>72</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>7</v>
+        <v>79</v>
       </c>
       <c r="F89" s="1" t="s">
         <v>36</v>

</xml_diff>

<commit_message>
Adding Customers Logic and Correcting Some CSS
</commit_message>
<xml_diff>
--- a/Planificacion/Base De Datos.xlsx
+++ b/Planificacion/Base De Datos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rayke\Documents\Programacion Web\Programacion 3\Proyecto Final\Reto-3-Grupo-J\Planificacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EC88281-F348-415D-BE5A-62A860755B20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19476057-0BB1-4809-8553-C4EBFC79991D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="7650" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="81">
   <si>
     <t>role_id</t>
   </si>
@@ -276,6 +276,9 @@
   </si>
   <si>
     <t>int8</t>
+  </si>
+  <si>
+    <t>image_url</t>
   </si>
 </sst>
 </file>
@@ -762,7 +765,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="D2:J97"/>
+  <dimension ref="D2:J99"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="4" max="4" width="17.81640625" bestFit="1" customWidth="1"/>
@@ -1646,23 +1649,23 @@
       </c>
     </row>
     <row r="62" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D62" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E62" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F62" s="1"/>
-      <c r="G62" s="1"/>
-      <c r="H62" s="1"/>
-      <c r="I62" s="1"/>
-      <c r="J62" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="D62" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="E62" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="F62" s="7"/>
+      <c r="G62" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="H62" s="7"/>
+      <c r="I62" s="7"/>
+      <c r="J62" s="7"/>
     </row>
     <row r="63" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D63" s="1" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="E63" s="1" t="s">
         <v>12</v>
@@ -1671,11 +1674,13 @@
       <c r="G63" s="1"/>
       <c r="H63" s="1"/>
       <c r="I63" s="1"/>
-      <c r="J63" s="1"/>
+      <c r="J63" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="64" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D64" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E64" s="1" t="s">
         <v>12</v>
@@ -1684,13 +1689,11 @@
       <c r="G64" s="1"/>
       <c r="H64" s="1"/>
       <c r="I64" s="1"/>
-      <c r="J64" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="J64" s="1"/>
     </row>
     <row r="65" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D65" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E65" s="1" t="s">
         <v>12</v>
@@ -1703,7 +1706,7 @@
     </row>
     <row r="66" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D66" s="1" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="E66" s="1" t="s">
         <v>12</v>
@@ -1712,171 +1715,169 @@
       <c r="G66" s="1"/>
       <c r="H66" s="1"/>
       <c r="I66" s="1"/>
-      <c r="J66" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="J66" s="1"/>
     </row>
     <row r="67" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D67" s="1" t="s">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F67" s="1"/>
       <c r="G67" s="1"/>
       <c r="H67" s="1"/>
       <c r="I67" s="1"/>
-      <c r="J67" s="1"/>
+      <c r="J67" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="68" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D68" s="1" t="s">
-        <v>4</v>
+        <v>80</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F68" s="1"/>
       <c r="G68" s="1"/>
-      <c r="H68" s="1" t="s">
-        <v>27</v>
-      </c>
+      <c r="H68" s="1"/>
       <c r="I68" s="1"/>
-      <c r="J68" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="J68" s="1"/>
     </row>
     <row r="69" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D69" s="1" t="s">
-        <v>23</v>
+        <v>57</v>
       </c>
       <c r="E69" s="1" t="s">
         <v>13</v>
       </c>
       <c r="F69" s="1"/>
       <c r="G69" s="1"/>
-      <c r="H69" s="1" t="s">
+      <c r="H69" s="1"/>
+      <c r="I69" s="1"/>
+      <c r="J69" s="1"/>
+    </row>
+    <row r="70" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D70" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E70" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F70" s="1"/>
+      <c r="G70" s="1"/>
+      <c r="H70" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="I69" s="1" t="s">
+      <c r="I70" s="1"/>
+      <c r="J70" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="71" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D71" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E71" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F71" s="1"/>
+      <c r="G71" s="1"/>
+      <c r="H71" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="I71" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="J69" s="1" t="s">
+      <c r="J71" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="71" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D71" s="17" t="s">
+    <row r="73" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D73" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="E71" s="17"/>
-      <c r="F71" s="17"/>
-      <c r="G71" s="17"/>
-      <c r="H71" s="17"/>
-      <c r="I71" s="17"/>
-      <c r="J71" s="17"/>
-    </row>
-    <row r="72" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D72" s="2" t="s">
+      <c r="E73" s="17"/>
+      <c r="F73" s="17"/>
+      <c r="G73" s="17"/>
+      <c r="H73" s="17"/>
+      <c r="I73" s="17"/>
+      <c r="J73" s="17"/>
+    </row>
+    <row r="74" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D74" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E72" s="3" t="s">
+      <c r="E74" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F72" s="3" t="s">
+      <c r="F74" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="G72" s="3" t="s">
+      <c r="G74" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H72" s="3" t="s">
+      <c r="H74" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="I72" s="3" t="s">
+      <c r="I74" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="J72" s="3" t="s">
+      <c r="J74" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="73" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D73" s="1" t="s">
+    <row r="75" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D75" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="E73" s="1" t="s">
+      <c r="E75" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="F73" s="1" t="s">
+      <c r="F75" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G73" s="1"/>
-      <c r="H73" s="1"/>
-      <c r="I73" s="1"/>
-      <c r="J73" s="1" t="s">
+      <c r="G75" s="1"/>
+      <c r="H75" s="1"/>
+      <c r="I75" s="1"/>
+      <c r="J75" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="74" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D74" s="8" t="s">
+    <row r="76" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D76" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="E74" s="8" t="s">
+      <c r="E76" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="F74" s="8"/>
-      <c r="G74" s="8" t="s">
+      <c r="F76" s="8"/>
+      <c r="G76" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="H74" s="8"/>
-      <c r="I74" s="8"/>
-      <c r="J74" s="8"/>
-    </row>
-    <row r="75" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D75" s="9" t="s">
+      <c r="H76" s="8"/>
+      <c r="I76" s="8"/>
+      <c r="J76" s="8"/>
+    </row>
+    <row r="77" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D77" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="E75" s="9" t="s">
+      <c r="E77" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="F75" s="9"/>
-      <c r="G75" s="9" t="s">
+      <c r="F77" s="9"/>
+      <c r="G77" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="H75" s="9"/>
-      <c r="I75" s="9"/>
-      <c r="J75" s="9"/>
-    </row>
-    <row r="76" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D76" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="E76" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F76" s="1"/>
-      <c r="G76" s="1"/>
-      <c r="H76" s="1"/>
-      <c r="I76" s="1"/>
-      <c r="J76" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="77" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D77" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="E77" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F77" s="1"/>
-      <c r="G77" s="1"/>
-      <c r="H77" s="1"/>
-      <c r="I77" s="1"/>
-      <c r="J77" s="1"/>
+      <c r="H77" s="9"/>
+      <c r="I77" s="9"/>
+      <c r="J77" s="9"/>
     </row>
     <row r="78" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D78" s="1" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="E78" s="1" t="s">
         <v>12</v>
@@ -1885,11 +1886,13 @@
       <c r="G78" s="1"/>
       <c r="H78" s="1"/>
       <c r="I78" s="1"/>
-      <c r="J78" s="1"/>
+      <c r="J78" s="1" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="79" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D79" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E79" s="1" t="s">
         <v>12</v>
@@ -1902,10 +1905,10 @@
     </row>
     <row r="80" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D80" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="F80" s="1"/>
       <c r="G80" s="1"/>
@@ -1915,10 +1918,10 @@
     </row>
     <row r="81" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D81" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="F81" s="1"/>
       <c r="G81" s="1"/>
@@ -1928,7 +1931,7 @@
     </row>
     <row r="82" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D82" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E82" s="1" t="s">
         <v>44</v>
@@ -1941,7 +1944,7 @@
     </row>
     <row r="83" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D83" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E83" s="1" t="s">
         <v>44</v>
@@ -1954,165 +1957,165 @@
     </row>
     <row r="84" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D84" s="1" t="s">
-        <v>4</v>
+        <v>66</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>13</v>
+        <v>44</v>
       </c>
       <c r="F84" s="1"/>
       <c r="G84" s="1"/>
-      <c r="H84" s="1" t="s">
-        <v>27</v>
-      </c>
+      <c r="H84" s="1"/>
       <c r="I84" s="1"/>
-      <c r="J84" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="J84" s="1"/>
     </row>
     <row r="85" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D85" s="1" t="s">
-        <v>23</v>
+        <v>67</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>13</v>
+        <v>44</v>
       </c>
       <c r="F85" s="1"/>
       <c r="G85" s="1"/>
-      <c r="H85" s="1" t="s">
+      <c r="H85" s="1"/>
+      <c r="I85" s="1"/>
+      <c r="J85" s="1"/>
+    </row>
+    <row r="86" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D86" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E86" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F86" s="1"/>
+      <c r="G86" s="1"/>
+      <c r="H86" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="I85" s="1" t="s">
+      <c r="I86" s="1"/>
+      <c r="J86" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="87" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D87" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E87" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F87" s="1"/>
+      <c r="G87" s="1"/>
+      <c r="H87" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="I87" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="J85" s="1" t="s">
+      <c r="J87" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="87" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D87" s="10" t="s">
+    <row r="89" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D89" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="E87" s="10"/>
-      <c r="F87" s="10"/>
-      <c r="G87" s="10"/>
-      <c r="H87" s="10"/>
-      <c r="I87" s="10"/>
-      <c r="J87" s="10"/>
-    </row>
-    <row r="88" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D88" s="2" t="s">
+      <c r="E89" s="10"/>
+      <c r="F89" s="10"/>
+      <c r="G89" s="10"/>
+      <c r="H89" s="10"/>
+      <c r="I89" s="10"/>
+      <c r="J89" s="10"/>
+    </row>
+    <row r="90" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D90" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E88" s="3" t="s">
+      <c r="E90" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F88" s="3" t="s">
+      <c r="F90" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="G88" s="3" t="s">
+      <c r="G90" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H88" s="3" t="s">
+      <c r="H90" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="I88" s="3" t="s">
+      <c r="I90" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="J88" s="3" t="s">
+      <c r="J90" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="89" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D89" s="1" t="s">
+    <row r="91" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D91" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E89" s="1" t="s">
+      <c r="E91" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="F89" s="1" t="s">
+      <c r="F91" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G89" s="1"/>
-      <c r="H89" s="1"/>
-      <c r="I89" s="1"/>
-      <c r="J89" s="1" t="s">
+      <c r="G91" s="1"/>
+      <c r="H91" s="1"/>
+      <c r="I91" s="1"/>
+      <c r="J91" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="90" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D90" s="8" t="s">
+    <row r="92" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D92" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="E90" s="8" t="s">
+      <c r="E92" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="F90" s="8"/>
-      <c r="G90" s="8" t="s">
+      <c r="F92" s="8"/>
+      <c r="G92" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="H90" s="8"/>
-      <c r="I90" s="8"/>
-      <c r="J90" s="8"/>
-    </row>
-    <row r="91" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D91" s="9" t="s">
+      <c r="H92" s="8"/>
+      <c r="I92" s="8"/>
+      <c r="J92" s="8"/>
+    </row>
+    <row r="93" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D93" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="E91" s="9" t="s">
+      <c r="E93" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="F91" s="9"/>
-      <c r="G91" s="9" t="s">
+      <c r="F93" s="9"/>
+      <c r="G93" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="H91" s="9"/>
-      <c r="I91" s="9"/>
-      <c r="J91" s="9"/>
-    </row>
-    <row r="92" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D92" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E92" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F92" s="1"/>
-      <c r="G92" s="1"/>
-      <c r="H92" s="1"/>
-      <c r="I92" s="1"/>
-      <c r="J92" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="93" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D93" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="E93" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="F93" s="1"/>
-      <c r="G93" s="1"/>
-      <c r="H93" s="1"/>
-      <c r="I93" s="1"/>
-      <c r="J93" s="1"/>
+      <c r="H93" s="9"/>
+      <c r="I93" s="9"/>
+      <c r="J93" s="9"/>
     </row>
     <row r="94" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D94" s="1" t="s">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="E94" s="1" t="s">
-        <v>44</v>
+        <v>7</v>
       </c>
       <c r="F94" s="1"/>
       <c r="G94" s="1"/>
       <c r="H94" s="1"/>
       <c r="I94" s="1"/>
-      <c r="J94" s="1"/>
+      <c r="J94" s="1" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="95" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D95" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E95" s="1" t="s">
         <v>44</v>
@@ -2125,50 +2128,76 @@
     </row>
     <row r="96" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D96" s="1" t="s">
-        <v>4</v>
+        <v>66</v>
       </c>
       <c r="E96" s="1" t="s">
-        <v>13</v>
+        <v>44</v>
       </c>
       <c r="F96" s="1"/>
       <c r="G96" s="1"/>
-      <c r="H96" s="1" t="s">
-        <v>27</v>
-      </c>
+      <c r="H96" s="1"/>
       <c r="I96" s="1"/>
-      <c r="J96" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="J96" s="1"/>
     </row>
     <row r="97" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D97" s="1" t="s">
-        <v>23</v>
+        <v>77</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>13</v>
+        <v>44</v>
       </c>
       <c r="F97" s="1"/>
       <c r="G97" s="1"/>
-      <c r="H97" s="1" t="s">
+      <c r="H97" s="1"/>
+      <c r="I97" s="1"/>
+      <c r="J97" s="1"/>
+    </row>
+    <row r="98" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D98" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E98" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F98" s="1"/>
+      <c r="G98" s="1"/>
+      <c r="H98" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="I97" s="1" t="s">
+      <c r="I98" s="1"/>
+      <c r="J98" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="99" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D99" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E99" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F99" s="1"/>
+      <c r="G99" s="1"/>
+      <c r="H99" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="I99" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="J97" s="1" t="s">
+      <c r="J99" s="1" t="s">
         <v>24</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="D87:J87"/>
+    <mergeCell ref="D89:J89"/>
     <mergeCell ref="D2:J2"/>
     <mergeCell ref="D9:J9"/>
     <mergeCell ref="D20:J20"/>
     <mergeCell ref="D31:J31"/>
     <mergeCell ref="D46:J46"/>
     <mergeCell ref="D59:J59"/>
-    <mergeCell ref="D71:J71"/>
+    <mergeCell ref="D73:J73"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Agregando Mas de 7 Horas De trabajo. Hahaha
</commit_message>
<xml_diff>
--- a/Planificacion/Base De Datos.xlsx
+++ b/Planificacion/Base De Datos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rayke\Documents\Programacion Web\Programacion 3\Proyecto Final\Reto-3-Grupo-J\Planificacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA3902F6-45F9-4E4D-9D3C-9D45647C4041}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5A687CE-C06A-49E6-B525-EA382658C79E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="19380" windowHeight="20970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="7650" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="90">
   <si>
     <t>role_id</t>
   </si>
@@ -306,9 +306,6 @@
   </si>
   <si>
     <t>Yes - deparments(department_id)</t>
-  </si>
-  <si>
-    <t>department_url</t>
   </si>
 </sst>
 </file>
@@ -474,7 +471,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -503,6 +500,15 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -525,18 +531,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -832,15 +826,15 @@
   </cols>
   <sheetData>
     <row r="2" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D2" s="11" t="s">
+      <c r="D2" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="11"/>
-      <c r="I2" s="11"/>
-      <c r="J2" s="11"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
+      <c r="J2" s="14"/>
     </row>
     <row r="3" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D3" s="2" t="s">
@@ -928,15 +922,15 @@
       </c>
     </row>
     <row r="9" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D9" s="12" t="s">
+      <c r="D9" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="12"/>
-      <c r="I9" s="12"/>
-      <c r="J9" s="12"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="15"/>
+      <c r="I9" s="15"/>
+      <c r="J9" s="15"/>
     </row>
     <row r="10" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D10" s="2" t="s">
@@ -1088,15 +1082,15 @@
       </c>
     </row>
     <row r="20" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D20" s="13" t="s">
+      <c r="D20" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="E20" s="13"/>
-      <c r="F20" s="13"/>
-      <c r="G20" s="13"/>
-      <c r="H20" s="13"/>
-      <c r="I20" s="13"/>
-      <c r="J20" s="13"/>
+      <c r="E20" s="16"/>
+      <c r="F20" s="16"/>
+      <c r="G20" s="16"/>
+      <c r="H20" s="16"/>
+      <c r="I20" s="16"/>
+      <c r="J20" s="16"/>
     </row>
     <row r="21" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D21" s="2" t="s">
@@ -1242,15 +1236,15 @@
       </c>
     </row>
     <row r="31" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D31" s="20" t="s">
+      <c r="D31" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="E31" s="20"/>
-      <c r="F31" s="20"/>
-      <c r="G31" s="20"/>
-      <c r="H31" s="20"/>
-      <c r="I31" s="20"/>
-      <c r="J31" s="20"/>
+      <c r="E31" s="12"/>
+      <c r="F31" s="12"/>
+      <c r="G31" s="12"/>
+      <c r="H31" s="12"/>
+      <c r="I31" s="12"/>
+      <c r="J31" s="12"/>
     </row>
     <row r="32" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D32" s="2" t="s">
@@ -1293,32 +1287,32 @@
       </c>
     </row>
     <row r="34" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D34" s="19" t="s">
+      <c r="D34" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E34" s="19" t="s">
+      <c r="E34" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="F34" s="19"/>
-      <c r="G34" s="19"/>
-      <c r="H34" s="19"/>
-      <c r="I34" s="19"/>
-      <c r="J34" s="19" t="s">
+      <c r="F34" s="1"/>
+      <c r="G34" s="1"/>
+      <c r="H34" s="1"/>
+      <c r="I34" s="1"/>
+      <c r="J34" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="35" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D35" s="19" t="s">
-        <v>90</v>
-      </c>
-      <c r="E35" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="F35" s="19"/>
-      <c r="G35" s="19"/>
-      <c r="H35" s="19"/>
-      <c r="I35" s="19"/>
-      <c r="J35" s="19"/>
+      <c r="D35" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F35" s="1"/>
+      <c r="G35" s="1"/>
+      <c r="H35" s="1"/>
+      <c r="I35" s="1"/>
+      <c r="J35" s="1"/>
     </row>
     <row r="36" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D36" s="1" t="s">
@@ -1357,15 +1351,15 @@
       </c>
     </row>
     <row r="39" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D39" s="14" t="s">
+      <c r="D39" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="E39" s="14"/>
-      <c r="F39" s="14"/>
-      <c r="G39" s="14"/>
-      <c r="H39" s="14"/>
-      <c r="I39" s="14"/>
-      <c r="J39" s="14"/>
+      <c r="E39" s="17"/>
+      <c r="F39" s="17"/>
+      <c r="G39" s="17"/>
+      <c r="H39" s="17"/>
+      <c r="I39" s="17"/>
+      <c r="J39" s="17"/>
     </row>
     <row r="40" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D40" s="2" t="s">
@@ -1541,19 +1535,19 @@
       </c>
     </row>
     <row r="51" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D51" s="21" t="s">
+      <c r="D51" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="E51" s="21" t="s">
+      <c r="E51" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="F51" s="21"/>
-      <c r="G51" s="21" t="s">
+      <c r="F51" s="10"/>
+      <c r="G51" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="H51" s="21"/>
-      <c r="I51" s="21"/>
-      <c r="J51" s="21" t="s">
+      <c r="H51" s="10"/>
+      <c r="I51" s="10"/>
+      <c r="J51" s="10" t="s">
         <v>16</v>
       </c>
     </row>
@@ -1607,15 +1601,15 @@
       </c>
     </row>
     <row r="57" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D57" s="15" t="s">
+      <c r="D57" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="E57" s="15"/>
-      <c r="F57" s="15"/>
-      <c r="G57" s="15"/>
-      <c r="H57" s="15"/>
-      <c r="I57" s="15"/>
-      <c r="J57" s="15"/>
+      <c r="E57" s="18"/>
+      <c r="F57" s="18"/>
+      <c r="G57" s="18"/>
+      <c r="H57" s="18"/>
+      <c r="I57" s="18"/>
+      <c r="J57" s="18"/>
     </row>
     <row r="58" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D58" s="2" t="s">
@@ -1795,15 +1789,15 @@
       </c>
     </row>
     <row r="70" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D70" s="16" t="s">
+      <c r="D70" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="E70" s="16"/>
-      <c r="F70" s="16"/>
-      <c r="G70" s="16"/>
-      <c r="H70" s="16"/>
-      <c r="I70" s="16"/>
-      <c r="J70" s="16"/>
+      <c r="E70" s="19"/>
+      <c r="F70" s="19"/>
+      <c r="G70" s="19"/>
+      <c r="H70" s="19"/>
+      <c r="I70" s="19"/>
+      <c r="J70" s="19"/>
     </row>
     <row r="71" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D71" s="2" t="s">
@@ -1994,15 +1988,15 @@
       </c>
     </row>
     <row r="84" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D84" s="17" t="s">
+      <c r="D84" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="E84" s="17"/>
-      <c r="F84" s="17"/>
-      <c r="G84" s="17"/>
-      <c r="H84" s="17"/>
-      <c r="I84" s="17"/>
-      <c r="J84" s="17"/>
+      <c r="E84" s="20"/>
+      <c r="F84" s="20"/>
+      <c r="G84" s="20"/>
+      <c r="H84" s="20"/>
+      <c r="I84" s="20"/>
+      <c r="J84" s="20"/>
     </row>
     <row r="85" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D85" s="2" t="s">
@@ -2221,15 +2215,15 @@
       </c>
     </row>
     <row r="100" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D100" s="10" t="s">
+      <c r="D100" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="E100" s="10"/>
-      <c r="F100" s="10"/>
-      <c r="G100" s="10"/>
-      <c r="H100" s="10"/>
-      <c r="I100" s="10"/>
-      <c r="J100" s="10"/>
+      <c r="E100" s="13"/>
+      <c r="F100" s="13"/>
+      <c r="G100" s="13"/>
+      <c r="H100" s="13"/>
+      <c r="I100" s="13"/>
+      <c r="J100" s="13"/>
     </row>
     <row r="101" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D101" s="2" t="s">
@@ -2394,15 +2388,15 @@
       </c>
     </row>
     <row r="112" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D112" s="18" t="s">
+      <c r="D112" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="E112" s="18"/>
-      <c r="F112" s="18"/>
-      <c r="G112" s="18"/>
-      <c r="H112" s="18"/>
-      <c r="I112" s="18"/>
-      <c r="J112" s="18"/>
+      <c r="E112" s="11"/>
+      <c r="F112" s="11"/>
+      <c r="G112" s="11"/>
+      <c r="H112" s="11"/>
+      <c r="I112" s="11"/>
+      <c r="J112" s="11"/>
     </row>
     <row r="113" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D113" s="2" t="s">

</xml_diff>

<commit_message>
Fixing Bugs and Issues with Orders and Profile
</commit_message>
<xml_diff>
--- a/Planificacion/Base De Datos.xlsx
+++ b/Planificacion/Base De Datos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rayke\Documents\Programacion Web\Programacion 3\Proyecto Final\Reto-3-Grupo-J\Planificacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5A687CE-C06A-49E6-B525-EA382658C79E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA9D046C-1108-4A9C-BA71-1D53A353408A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="7650" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="90">
   <si>
     <t>role_id</t>
   </si>
@@ -1854,7 +1854,9 @@
       </c>
       <c r="H73" s="7"/>
       <c r="I73" s="7"/>
-      <c r="J73" s="7"/>
+      <c r="J73" s="7" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="74" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D74" s="1" t="s">

</xml_diff>